<commit_message>
fix: stabilize permissions, resolve Next.js 16 regressions & build errors
</commit_message>
<xml_diff>
--- a/public/Seat Location.xlsx
+++ b/public/Seat Location.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chandan Kushwaha\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Project IT\MAMS\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76B976FA-0B0B-4D77-8C53-22E6C1DB375C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7E7C8E8-DA8F-431F-9AF1-15D119E52487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F8B282AC-972D-4C21-B6C6-E3DDE1FD64E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F8B282AC-972D-4C21-B6C6-E3DDE1FD64E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="441">
   <si>
     <t>MPL-WS001</t>
   </si>
@@ -1272,6 +1272,96 @@
   </si>
   <si>
     <t>CEO</t>
+  </si>
+  <si>
+    <t>IT-WS001</t>
+  </si>
+  <si>
+    <t>IT-WS002</t>
+  </si>
+  <si>
+    <t>IT-WS003</t>
+  </si>
+  <si>
+    <t>IT-WS004</t>
+  </si>
+  <si>
+    <t>IT-WS005</t>
+  </si>
+  <si>
+    <t>IT-WS006</t>
+  </si>
+  <si>
+    <t>IT-WS007</t>
+  </si>
+  <si>
+    <t>IT-WS008</t>
+  </si>
+  <si>
+    <t>IT-WS009</t>
+  </si>
+  <si>
+    <t>IT-WS010</t>
+  </si>
+  <si>
+    <t>Admin-WS01</t>
+  </si>
+  <si>
+    <t>Admin-WS02</t>
+  </si>
+  <si>
+    <t>Admin-WS03</t>
+  </si>
+  <si>
+    <t>Admin-WS04</t>
+  </si>
+  <si>
+    <t>Admin-WS05</t>
+  </si>
+  <si>
+    <t>Admin-WS06</t>
+  </si>
+  <si>
+    <t>Admin-WS07</t>
+  </si>
+  <si>
+    <t>Admin-WS08</t>
+  </si>
+  <si>
+    <t>Admin-WS09</t>
+  </si>
+  <si>
+    <t>Admin-WS10</t>
+  </si>
+  <si>
+    <t>Legal-WS01</t>
+  </si>
+  <si>
+    <t>Legal-WS02</t>
+  </si>
+  <si>
+    <t>Legal-WS03</t>
+  </si>
+  <si>
+    <t>Legal-WS04</t>
+  </si>
+  <si>
+    <t>Legal-WS05</t>
+  </si>
+  <si>
+    <t>Legal-WS06</t>
+  </si>
+  <si>
+    <t>Legal-WS07</t>
+  </si>
+  <si>
+    <t>Legal-WS08</t>
+  </si>
+  <si>
+    <t>Legal-WS09</t>
+  </si>
+  <si>
+    <t>Legal-WS10</t>
   </si>
 </sst>
 </file>
@@ -1655,15 +1745,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86AD768C-7E9A-4D9A-B83E-40B4103176CD}">
-  <dimension ref="A1:G175"/>
+  <dimension ref="A1:P175"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1965,7 +2063,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>38</v>
       </c>
@@ -1979,7 +2077,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -1993,7 +2091,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -2007,7 +2105,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -2021,7 +2119,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>42</v>
       </c>
@@ -2035,7 +2133,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -2049,7 +2147,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>44</v>
       </c>
@@ -2063,7 +2161,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>45</v>
       </c>
@@ -2077,7 +2175,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>46</v>
       </c>
@@ -2091,7 +2189,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>47</v>
       </c>
@@ -2105,7 +2203,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>48</v>
       </c>
@@ -2119,7 +2217,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>49</v>
       </c>
@@ -2133,7 +2231,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>50</v>
       </c>
@@ -2147,7 +2245,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>51</v>
       </c>
@@ -2160,8 +2258,35 @@
       <c r="E30" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H30" t="s">
+        <v>374</v>
+      </c>
+      <c r="I30" t="s">
+        <v>375</v>
+      </c>
+      <c r="J30" t="s">
+        <v>376</v>
+      </c>
+      <c r="K30" t="s">
+        <v>377</v>
+      </c>
+      <c r="L30" t="s">
+        <v>393</v>
+      </c>
+      <c r="M30" t="s">
+        <v>395</v>
+      </c>
+      <c r="N30" t="s">
+        <v>396</v>
+      </c>
+      <c r="O30" t="s">
+        <v>397</v>
+      </c>
+      <c r="P30" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>52</v>
       </c>
@@ -2174,8 +2299,17 @@
       <c r="E31" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H31" t="s">
+        <v>411</v>
+      </c>
+      <c r="I31" t="s">
+        <v>421</v>
+      </c>
+      <c r="J31" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>53</v>
       </c>
@@ -2188,8 +2322,17 @@
       <c r="E32" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H32" t="s">
+        <v>412</v>
+      </c>
+      <c r="I32" t="s">
+        <v>422</v>
+      </c>
+      <c r="J32" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>54</v>
       </c>
@@ -2202,8 +2345,17 @@
       <c r="E33" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H33" t="s">
+        <v>413</v>
+      </c>
+      <c r="I33" t="s">
+        <v>423</v>
+      </c>
+      <c r="J33" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>55</v>
       </c>
@@ -2216,8 +2368,17 @@
       <c r="E34" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H34" t="s">
+        <v>414</v>
+      </c>
+      <c r="I34" t="s">
+        <v>424</v>
+      </c>
+      <c r="J34" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>56</v>
       </c>
@@ -2230,8 +2391,17 @@
       <c r="E35" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H35" t="s">
+        <v>415</v>
+      </c>
+      <c r="I35" t="s">
+        <v>425</v>
+      </c>
+      <c r="J35" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>57</v>
       </c>
@@ -2244,8 +2414,17 @@
       <c r="E36" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H36" t="s">
+        <v>416</v>
+      </c>
+      <c r="I36" t="s">
+        <v>426</v>
+      </c>
+      <c r="J36" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>58</v>
       </c>
@@ -2255,8 +2434,17 @@
       <c r="E37" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H37" t="s">
+        <v>417</v>
+      </c>
+      <c r="I37" t="s">
+        <v>427</v>
+      </c>
+      <c r="J37" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>59</v>
       </c>
@@ -2266,8 +2454,17 @@
       <c r="E38" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H38" t="s">
+        <v>418</v>
+      </c>
+      <c r="I38" t="s">
+        <v>428</v>
+      </c>
+      <c r="J38" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>60</v>
       </c>
@@ -2277,8 +2474,17 @@
       <c r="E39" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H39" t="s">
+        <v>419</v>
+      </c>
+      <c r="I39" t="s">
+        <v>429</v>
+      </c>
+      <c r="J39" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>61</v>
       </c>
@@ -2288,8 +2494,17 @@
       <c r="E40" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H40" t="s">
+        <v>420</v>
+      </c>
+      <c r="I40" t="s">
+        <v>430</v>
+      </c>
+      <c r="J40" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>62</v>
       </c>
@@ -2300,7 +2515,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>63</v>
       </c>
@@ -2311,7 +2526,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>64</v>
       </c>
@@ -2322,7 +2537,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>65</v>
       </c>
@@ -2333,7 +2548,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>66</v>
       </c>
@@ -2344,7 +2559,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>67</v>
       </c>
@@ -2355,7 +2570,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>68</v>
       </c>
@@ -2366,7 +2581,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>69</v>
       </c>

</xml_diff>